<commit_message>
feat: expand synthetic tariff data and mock sources
</commit_message>
<xml_diff>
--- a/data/input/tariff_packs.xlsx
+++ b/data/input/tariff_packs.xlsx
@@ -135,8 +135,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TariffPacks" displayName="TariffPacks" ref="A1:M16" headerRowCount="1">
-  <autoFilter ref="A1:M16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TariffPacks" displayName="TariffPacks" ref="A1:M29" headerRowCount="1">
+  <autoFilter ref="A1:M29"/>
   <tableColumns count="13">
     <tableColumn id="1" name="pack_id"/>
     <tableColumn id="2" name="pack_name"/>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -460,7 +460,7 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,6 +546,9 @@
           <t>Youth</t>
         </is>
       </c>
+      <c r="D2" t="n">
+        <v>11.9</v>
+      </c>
       <c r="E2" t="n">
         <v>30</v>
       </c>
@@ -575,12 +578,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>old email pre-release price</t>
+          <t>old draft price and activation code</t>
         </is>
       </c>
     </row>
@@ -601,13 +604,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>24.9</v>
+        <v>29.9</v>
       </c>
       <c r="E3" t="n">
         <v>30</v>
       </c>
       <c r="F3" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G3" t="n">
         <v>800</v>
@@ -632,12 +635,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>old confluence name</t>
+          <t>old pack name should be renamed</t>
         </is>
       </c>
     </row>
@@ -649,12 +652,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Night Internet Pack 5GB</t>
+          <t>Night Owl 5GB</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Postpaid</t>
+          <t>Prepaid</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -672,14 +675,9 @@
       <c r="H4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>5555</t>
-        </is>
-      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -689,12 +687,12 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>tariff eligibility mismatch</t>
+          <t>missing final activation code</t>
         </is>
       </c>
     </row>
@@ -706,34 +704,37 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Student Social 3GB</t>
+          <t>Roaming Lite 1GB</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Youth</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5.9</v>
+        <v>7.5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>7</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="H5" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>*321*3#</t>
+          <t>*123*77#</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -743,12 +744,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>missing validity</t>
+          <t>draft minutes</t>
         </is>
       </c>
     </row>
@@ -760,32 +761,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Weekend Unlimited</t>
+          <t>Student Social 3GB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prepaid</t>
+          <t>Youth</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>9.9</v>
+        <v>5.9</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>999</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>*888#</t>
+          <t>*321*3#</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -800,12 +801,12 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>status may be retired</t>
+          <t>discontinued pack still active</t>
         </is>
       </c>
     </row>
@@ -817,32 +818,37 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Data Boost 15GB</t>
+          <t>Family Data 18GB</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Data-only</t>
+          <t>Postpaid</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>14.9</v>
+        <v>21.9</v>
       </c>
       <c r="E7" t="n">
         <v>30</v>
       </c>
       <c r="F7" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>200</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>*456*18#</t>
+        </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -852,12 +858,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>missing activation code and old data value</t>
+          <t>replaced by Family Share 20GB</t>
         </is>
       </c>
     </row>
@@ -869,37 +875,37 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Roaming Lite 1GB</t>
+          <t>Executive Voice 1000</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.5</v>
+        <v>19.9</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>30</v>
+        <v>1000</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>*901*1#</t>
+          <t>*700*1000#</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -909,12 +915,12 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>suspiciously low roaming price</t>
+          <t>correct row</t>
         </is>
       </c>
     </row>
@@ -926,32 +932,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Family Share 40GB</t>
+          <t>SME Connect 15GB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Postpaid</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>39.9</v>
+        <v>18.9</v>
       </c>
       <c r="E9" t="n">
         <v>30</v>
       </c>
       <c r="F9" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="G9" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="H9" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>*444*40#</t>
+          <t>*345*15#</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -961,7 +967,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -978,22 +984,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Promo Flash 2GB</t>
+          <t>Enterprise Data 50GB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Prepaid</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2.9</v>
+        <v>49.9</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -1001,29 +1007,24 @@
       <c r="H10" t="n">
         <v>0</v>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>*222*2#</t>
-        </is>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>inactive</t>
+          <t>active</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>conflicting status</t>
+          <t>missing activation code</t>
         </is>
       </c>
     </row>
@@ -1035,37 +1036,37 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mega Stream 50GB</t>
+          <t>Weekend Turbo 8GB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Data-only</t>
+          <t>Prepaid</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>120</v>
+        <v>0.4</v>
       </c>
       <c r="E11" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="F11" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="G11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>*777*50#</t>
+          <t>*888*8#</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1075,12 +1076,12 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2025-12-10</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>old source note and voice minutes mismatch</t>
+          <t>suspiciously low local price</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1093,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YouthMax 10GB</t>
+          <t>Social Mix 4GB</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1101,28 +1102,25 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="E12" t="n">
-        <v>30</v>
+        <v>6.9</v>
       </c>
       <c r="F12" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G12" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="H12" t="n">
         <v>100</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>*123*10#</t>
+          <t>*222*4#</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1132,12 +1130,12 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>duplicate pack name for review</t>
+          <t>missing validity</t>
         </is>
       </c>
     </row>
@@ -1149,52 +1147,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ultra Roaming 5GB</t>
+          <t>Data Boost 2GB</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Prepaid</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>149.9</v>
+        <v>2.9</v>
       </c>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G13" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>*909*5#</t>
+          <t>*222*2#</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>active</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>suspiciously high roaming price</t>
+          <t>missing status</t>
         </is>
       </c>
     </row>
@@ -1206,32 +1199,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Business Pro Plus</t>
+          <t>YouthMax 10GB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Youth</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>29.9</v>
+        <v>12.9</v>
       </c>
       <c r="E14" t="n">
         <v>30</v>
       </c>
       <c r="F14" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="H14" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>*234*25#</t>
+          <t>*123*10#</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1246,12 +1239,12 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>current approved name</t>
+          <t>duplicate good row</t>
         </is>
       </c>
     </row>
@@ -1263,37 +1256,34 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Micro Data 500MB</t>
+          <t>Roaming Max 5GB</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Data-only</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>0.2</v>
+          <t>Travel</t>
+        </is>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F15" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>*500#</t>
+          <t>*909*5#</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1303,12 +1293,12 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>suspiciously low local price</t>
+          <t>missing roaming price</t>
         </is>
       </c>
     </row>
@@ -1320,52 +1310,793 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Voice Plus 100</t>
+          <t>Business Pro Plus</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Data-only</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6.9</v>
+        <v>29.9</v>
       </c>
       <c r="E16" t="n">
         <v>30</v>
       </c>
       <c r="F16" t="n">
+        <v>25</v>
+      </c>
+      <c r="G16" t="n">
+        <v>800</v>
+      </c>
+      <c r="H16" t="n">
+        <v>200</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>*234*25#</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>correct row</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PK016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Night Owl 5GB</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Prepaid</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>*123*50#</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>old activation code</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PK017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Family Share 20GB</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Postpaid</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="E18" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" t="n">
+        <v>20</v>
+      </c>
+      <c r="G18" t="n">
+        <v>500</v>
+      </c>
+      <c r="H18" t="n">
+        <v>200</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>*456*20#</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>correct replacement row</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PK018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Enterprise Data 50GB</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="E19" t="n">
+        <v>30</v>
+      </c>
+      <c r="F19" t="n">
+        <v>50</v>
+      </c>
+      <c r="G19" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>*909*50#</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>data-only pack has unexpected minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PK019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SME Connect 15GB</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="E20" t="n">
+        <v>30</v>
+      </c>
+      <c r="F20" t="n">
+        <v>15</v>
+      </c>
+      <c r="G20" t="n">
+        <v>500</v>
+      </c>
+      <c r="H20" t="n">
+        <v>100</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>34515</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>invalid activation format</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PK020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roaming Lite 1GB</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E21" t="n">
+        <v>7</v>
+      </c>
+      <c r="F21" t="n">
         <v>1</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G21" t="n">
+        <v>20</v>
+      </c>
+      <c r="H21" t="n">
+        <v>10</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>*123*77#</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>duplicate correct roaming row</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PK021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Youth Weekend 6GB</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Youth</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="E22" t="n">
+        <v>7</v>
+      </c>
+      <c r="F22" t="n">
+        <v>6</v>
+      </c>
+      <c r="G22" t="n">
+        <v>50</v>
+      </c>
+      <c r="H22" t="n">
+        <v>50</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>*123*6#</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>good row not in conflict set</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PK022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Data Mini 1GB</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Prepaid</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>*101*1#</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>good low-cost row</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PK023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Executive Voice 1000</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="E24" t="n">
+        <v>30</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H24" t="n">
         <v>100</v>
       </c>
-      <c r="H16" t="n">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>*700*1000#</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>stale duplicate row</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PK024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Roaming Max 5GB</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>139.9</v>
+      </c>
+      <c r="E25" t="n">
+        <v>14</v>
+      </c>
+      <c r="F25" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" t="n">
+        <v>60</v>
+      </c>
+      <c r="H25" t="n">
+        <v>20</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>*909*5#</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>suspiciously high roaming price</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PK025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Social Mix 4GB</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Prepaid</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E26" t="n">
+        <v>14</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4</v>
+      </c>
+      <c r="G26" t="n">
         <v>100</v>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>*600*100#</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>tariff name mismatch and stale update</t>
+      <c r="H26" t="n">
+        <v>100</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>*222*4#</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>correct duplicate for comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PK026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Family Data 18GB</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Postpaid</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="E27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F27" t="n">
+        <v>18</v>
+      </c>
+      <c r="G27" t="n">
+        <v>400</v>
+      </c>
+      <c r="H27" t="n">
+        <v>200</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>*456*18#</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>inactive</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>old inactive replacement row</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PK027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Corporate Flex 30GB</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="E28" t="n">
+        <v>30</v>
+      </c>
+      <c r="F28" t="n">
+        <v>30</v>
+      </c>
+      <c r="G28" t="n">
+        <v>700</v>
+      </c>
+      <c r="H28" t="n">
+        <v>300</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>*789*30#</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>good business row</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PK028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Kids Safe 2GB</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Youth</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E29" t="n">
+        <v>30</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" t="n">
+        <v>50</v>
+      </c>
+      <c r="H29" t="n">
+        <v>50</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>*555*2#</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>good youth row</t>
         </is>
       </c>
     </row>

</xml_diff>